<commit_message>
Refactored and part working
RTC working well
Outputting 32KHz and saving time, etc
Deep sleep after initial time display
wake up with any button (inc reset!)
Simply displays time and goes to sleep again
80uA in deep sleep with test circuit
Debug output either to JTAG or UART at the mo - not sure why
EXT LP clock not detected ... clk: 32 kHz clock not found, switching to internal 150 kHz oscillator
</commit_message>
<xml_diff>
--- a/WordyFW/docs/20210115 Low Power Calculations.xlsx
+++ b/WordyFW/docs/20210115 Low Power Calculations.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\home\rob\rdev\WordyWatch\WordyFW\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02889DCB-A7EA-4F1D-A6C9-AB468CAF4312}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA5B01A8-D725-47B1-8683-D0D13394A5AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="390" yWindow="390" windowWidth="26250" windowHeight="13680" xr2:uid="{33FCFB16-DC53-4F12-BCE5-79061AEDC628}"/>
+    <workbookView xWindow="1560" yWindow="1560" windowWidth="26250" windowHeight="13680" xr2:uid="{33FCFB16-DC53-4F12-BCE5-79061AEDC628}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -169,11 +169,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -517,7 +516,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="3" t="s">
         <v>29</v>
       </c>
     </row>
@@ -755,7 +754,7 @@
       <c r="C16" s="1"/>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A17" s="4" t="s">
+      <c r="A17" s="3" t="s">
         <v>26</v>
       </c>
       <c r="C17" s="1"/>
@@ -793,7 +792,7 @@
         <f>E19*$D$19</f>
         <v>1.1797101449275365</v>
       </c>
-      <c r="G19" s="3">
+      <c r="G19">
         <v>1.2529999999999999</v>
       </c>
       <c r="H19">
@@ -814,7 +813,7 @@
         <f t="shared" ref="F20:F21" si="3">E20*$D$19</f>
         <v>1.0521739130434784</v>
       </c>
-      <c r="G20" s="3">
+      <c r="G20">
         <v>1.19</v>
       </c>
       <c r="H20">
@@ -829,7 +828,7 @@
         <f t="shared" si="3"/>
         <v>0.95652173913043481</v>
       </c>
-      <c r="G21" s="3">
+      <c r="G21">
         <v>1.0649999999999999</v>
       </c>
       <c r="H21">
@@ -837,7 +836,7 @@
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A23" s="4" t="s">
+      <c r="A23" s="3" t="s">
         <v>12</v>
       </c>
     </row>
@@ -863,22 +862,22 @@
         <v>13</v>
       </c>
       <c r="C25" s="1">
-        <v>2200000</v>
+        <v>4700000</v>
       </c>
       <c r="D25">
         <v>2.5</v>
       </c>
-      <c r="E25" s="3">
+      <c r="E25">
         <f>D25*$C$29</f>
-        <v>0.78125</v>
-      </c>
-      <c r="F25" s="3">
+        <v>0.79710144927536231</v>
+      </c>
+      <c r="F25">
         <f>D25*$C$30</f>
-        <v>1.4814814814814814</v>
+        <v>1.7427497314715359</v>
       </c>
       <c r="G25" s="1">
         <f>D25/$C$32</f>
-        <v>7.8125000000000004E-7</v>
+        <v>3.6231884057971015E-7</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
@@ -886,22 +885,22 @@
         <v>14</v>
       </c>
       <c r="C26" s="1">
-        <v>1000000</v>
+        <v>2200000</v>
       </c>
       <c r="D26">
         <v>2.6</v>
       </c>
-      <c r="E26" s="3">
+      <c r="E26">
         <f t="shared" ref="E26:E45" si="4">D26*$C$29</f>
-        <v>0.8125</v>
-      </c>
-      <c r="F26" s="3">
+        <v>0.82898550724637676</v>
+      </c>
+      <c r="F26">
         <f t="shared" ref="F26:F45" si="5">D26*$C$30</f>
-        <v>1.5407407407407407</v>
+        <v>1.8124597207303974</v>
       </c>
       <c r="G26" s="1">
         <f t="shared" ref="G26:G45" si="6">D26/$C$32</f>
-        <v>8.1250000000000006E-7</v>
+        <v>3.7681159420289855E-7</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
@@ -909,39 +908,39 @@
         <v>15</v>
       </c>
       <c r="C27" s="1">
-        <v>1000000</v>
+        <v>1200000</v>
       </c>
       <c r="D27">
         <v>2.7</v>
       </c>
-      <c r="E27" s="3">
-        <f t="shared" si="4"/>
-        <v>0.84375</v>
-      </c>
-      <c r="F27" s="3">
-        <f t="shared" si="5"/>
-        <v>1.6</v>
+      <c r="E27">
+        <f t="shared" si="4"/>
+        <v>0.86086956521739133</v>
+      </c>
+      <c r="F27">
+        <f t="shared" si="5"/>
+        <v>1.8821697099892589</v>
       </c>
       <c r="G27" s="1">
         <f t="shared" si="6"/>
-        <v>8.4375000000000007E-7</v>
+        <v>3.91304347826087E-7</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="D28">
         <v>2.8</v>
       </c>
-      <c r="E28" s="3">
-        <f t="shared" si="4"/>
-        <v>0.875</v>
-      </c>
-      <c r="F28" s="3">
-        <f t="shared" si="5"/>
-        <v>1.659259259259259</v>
+      <c r="E28">
+        <f t="shared" si="4"/>
+        <v>0.89275362318840568</v>
+      </c>
+      <c r="F28">
+        <f t="shared" si="5"/>
+        <v>1.9518796992481202</v>
       </c>
       <c r="G28" s="1">
         <f t="shared" si="6"/>
-        <v>8.7499999999999999E-7</v>
+        <v>4.0579710144927534E-7</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
@@ -950,22 +949,22 @@
       </c>
       <c r="C29" s="1">
         <f>C26/(C26+C25)</f>
-        <v>0.3125</v>
+        <v>0.3188405797101449</v>
       </c>
       <c r="D29">
         <v>2.9</v>
       </c>
-      <c r="E29" s="3">
-        <f t="shared" si="4"/>
-        <v>0.90625</v>
-      </c>
-      <c r="F29" s="3">
-        <f t="shared" si="5"/>
-        <v>1.7185185185185183</v>
+      <c r="E29">
+        <f t="shared" si="4"/>
+        <v>0.92463768115942013</v>
+      </c>
+      <c r="F29">
+        <f t="shared" si="5"/>
+        <v>2.0215896885069817</v>
       </c>
       <c r="G29" s="1">
         <f t="shared" si="6"/>
-        <v>9.0625000000000001E-7</v>
+        <v>4.2028985507246374E-7</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
@@ -974,39 +973,39 @@
       </c>
       <c r="C30" s="1">
         <f>C26/((C25*C27)/(C25+C27)+C26)</f>
-        <v>0.59259259259259256</v>
+        <v>0.69709989258861438</v>
       </c>
       <c r="D30">
         <v>3</v>
       </c>
-      <c r="E30" s="3">
-        <f t="shared" si="4"/>
-        <v>0.9375</v>
-      </c>
-      <c r="F30" s="3">
-        <f t="shared" si="5"/>
-        <v>1.7777777777777777</v>
+      <c r="E30">
+        <f t="shared" si="4"/>
+        <v>0.9565217391304347</v>
+      </c>
+      <c r="F30">
+        <f t="shared" si="5"/>
+        <v>2.0912996777658432</v>
       </c>
       <c r="G30" s="1">
         <f t="shared" si="6"/>
-        <v>9.3750000000000002E-7</v>
+        <v>4.3478260869565219E-7</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="D31">
         <v>3.1</v>
       </c>
-      <c r="E31" s="3">
-        <f t="shared" si="4"/>
-        <v>0.96875</v>
-      </c>
-      <c r="F31" s="3">
-        <f t="shared" si="5"/>
-        <v>1.837037037037037</v>
+      <c r="E31">
+        <f t="shared" si="4"/>
+        <v>0.98840579710144927</v>
+      </c>
+      <c r="F31">
+        <f t="shared" si="5"/>
+        <v>2.1610096670247048</v>
       </c>
       <c r="G31" s="1">
         <f t="shared" si="6"/>
-        <v>9.6875000000000004E-7</v>
+        <v>4.4927536231884059E-7</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
@@ -1015,243 +1014,243 @@
       </c>
       <c r="C32" s="1">
         <f>C25+C26</f>
-        <v>3200000</v>
+        <v>6900000</v>
       </c>
       <c r="D32">
         <v>3.2</v>
       </c>
-      <c r="E32" s="3">
-        <f t="shared" si="4"/>
-        <v>1</v>
-      </c>
-      <c r="F32" s="3">
-        <f t="shared" si="5"/>
-        <v>1.8962962962962964</v>
+      <c r="E32">
+        <f t="shared" si="4"/>
+        <v>1.0202898550724637</v>
+      </c>
+      <c r="F32">
+        <f t="shared" si="5"/>
+        <v>2.2307196562835663</v>
       </c>
       <c r="G32" s="1">
         <f t="shared" si="6"/>
-        <v>9.9999999999999995E-7</v>
+        <v>4.6376811594202904E-7</v>
       </c>
     </row>
     <row r="33" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D33">
         <v>3.3</v>
       </c>
-      <c r="E33" s="3">
-        <f t="shared" si="4"/>
-        <v>1.03125</v>
-      </c>
-      <c r="F33" s="3">
-        <f t="shared" si="5"/>
-        <v>1.9555555555555553</v>
+      <c r="E33">
+        <f t="shared" si="4"/>
+        <v>1.0521739130434782</v>
+      </c>
+      <c r="F33">
+        <f t="shared" si="5"/>
+        <v>2.3004296455424273</v>
       </c>
       <c r="G33" s="1">
         <f t="shared" si="6"/>
-        <v>1.0312499999999999E-6</v>
+        <v>4.7826086956521733E-7</v>
       </c>
     </row>
     <row r="34" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D34">
         <v>3.4</v>
       </c>
-      <c r="E34" s="3">
-        <f t="shared" si="4"/>
-        <v>1.0625</v>
-      </c>
-      <c r="F34" s="3">
-        <f t="shared" si="5"/>
-        <v>2.0148148148148146</v>
+      <c r="E34">
+        <f t="shared" si="4"/>
+        <v>1.0840579710144926</v>
+      </c>
+      <c r="F34">
+        <f t="shared" si="5"/>
+        <v>2.3701396348012889</v>
       </c>
       <c r="G34" s="1">
         <f t="shared" si="6"/>
-        <v>1.0625E-6</v>
+        <v>4.9275362318840583E-7</v>
       </c>
     </row>
     <row r="35" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D35">
         <v>3.5</v>
       </c>
-      <c r="E35" s="3">
-        <f t="shared" si="4"/>
-        <v>1.09375</v>
-      </c>
-      <c r="F35" s="3">
-        <f t="shared" si="5"/>
-        <v>2.074074074074074</v>
+      <c r="E35">
+        <f t="shared" si="4"/>
+        <v>1.1159420289855071</v>
+      </c>
+      <c r="F35">
+        <f t="shared" si="5"/>
+        <v>2.4398496240601504</v>
       </c>
       <c r="G35" s="1">
         <f t="shared" si="6"/>
-        <v>1.0937499999999999E-6</v>
+        <v>5.0724637681159423E-7</v>
       </c>
     </row>
     <row r="36" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D36">
         <v>3.6</v>
       </c>
-      <c r="E36" s="3">
-        <f t="shared" si="4"/>
-        <v>1.125</v>
-      </c>
-      <c r="F36" s="3">
-        <f t="shared" si="5"/>
-        <v>2.1333333333333333</v>
+      <c r="E36">
+        <f t="shared" si="4"/>
+        <v>1.1478260869565218</v>
+      </c>
+      <c r="F36">
+        <f t="shared" si="5"/>
+        <v>2.5095596133190119</v>
       </c>
       <c r="G36" s="1">
         <f t="shared" si="6"/>
-        <v>1.125E-6</v>
+        <v>5.2173913043478263E-7</v>
       </c>
     </row>
     <row r="37" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D37">
         <v>3.7</v>
       </c>
-      <c r="E37" s="3">
-        <f t="shared" si="4"/>
-        <v>1.15625</v>
-      </c>
-      <c r="F37" s="3">
-        <f t="shared" si="5"/>
-        <v>2.1925925925925926</v>
+      <c r="E37">
+        <f t="shared" si="4"/>
+        <v>1.1797101449275362</v>
+      </c>
+      <c r="F37">
+        <f t="shared" si="5"/>
+        <v>2.5792696025778734</v>
       </c>
       <c r="G37" s="1">
         <f t="shared" si="6"/>
-        <v>1.1562500000000002E-6</v>
+        <v>5.3623188405797102E-7</v>
       </c>
     </row>
     <row r="38" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D38">
         <v>3.8</v>
       </c>
-      <c r="E38" s="3">
-        <f t="shared" si="4"/>
-        <v>1.1875</v>
-      </c>
-      <c r="F38" s="3">
-        <f t="shared" si="5"/>
-        <v>2.2518518518518515</v>
+      <c r="E38">
+        <f t="shared" si="4"/>
+        <v>1.2115942028985505</v>
+      </c>
+      <c r="F38">
+        <f t="shared" si="5"/>
+        <v>2.6489795918367345</v>
       </c>
       <c r="G38" s="1">
         <f t="shared" si="6"/>
-        <v>1.1874999999999999E-6</v>
+        <v>5.5072463768115942E-7</v>
       </c>
     </row>
     <row r="39" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D39">
         <v>3.9</v>
       </c>
-      <c r="E39" s="3">
-        <f t="shared" si="4"/>
-        <v>1.21875</v>
-      </c>
-      <c r="F39" s="3">
-        <f t="shared" si="5"/>
-        <v>2.3111111111111109</v>
+      <c r="E39">
+        <f t="shared" si="4"/>
+        <v>1.2434782608695651</v>
+      </c>
+      <c r="F39">
+        <f t="shared" si="5"/>
+        <v>2.718689581095596</v>
       </c>
       <c r="G39" s="1">
         <f t="shared" si="6"/>
-        <v>1.21875E-6</v>
+        <v>5.6521739130434782E-7</v>
       </c>
     </row>
     <row r="40" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D40">
         <v>4</v>
       </c>
-      <c r="E40" s="3">
-        <f t="shared" si="4"/>
-        <v>1.25</v>
-      </c>
-      <c r="F40" s="3">
-        <f t="shared" si="5"/>
-        <v>2.3703703703703702</v>
+      <c r="E40">
+        <f t="shared" si="4"/>
+        <v>1.2753623188405796</v>
+      </c>
+      <c r="F40">
+        <f t="shared" si="5"/>
+        <v>2.7883995703544575</v>
       </c>
       <c r="G40" s="1">
         <f t="shared" si="6"/>
-        <v>1.2500000000000001E-6</v>
+        <v>5.7971014492753622E-7</v>
       </c>
     </row>
     <row r="41" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D41">
         <v>4.0999999999999996</v>
       </c>
-      <c r="E41" s="3">
-        <f t="shared" si="4"/>
-        <v>1.28125</v>
-      </c>
-      <c r="F41" s="3">
-        <f t="shared" si="5"/>
-        <v>2.4296296296296291</v>
+      <c r="E41">
+        <f t="shared" si="4"/>
+        <v>1.3072463768115941</v>
+      </c>
+      <c r="F41">
+        <f t="shared" si="5"/>
+        <v>2.8581095596133186</v>
       </c>
       <c r="G41" s="1">
         <f t="shared" si="6"/>
-        <v>1.2812499999999998E-6</v>
+        <v>5.9420289855072461E-7</v>
       </c>
     </row>
     <row r="42" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D42">
         <v>4.2</v>
       </c>
-      <c r="E42" s="3">
-        <f t="shared" si="4"/>
-        <v>1.3125</v>
-      </c>
-      <c r="F42" s="3">
-        <f t="shared" si="5"/>
-        <v>2.4888888888888889</v>
+      <c r="E42">
+        <f t="shared" si="4"/>
+        <v>1.3391304347826087</v>
+      </c>
+      <c r="F42">
+        <f t="shared" si="5"/>
+        <v>2.9278195488721805</v>
       </c>
       <c r="G42" s="1">
         <f t="shared" si="6"/>
-        <v>1.3125000000000001E-6</v>
+        <v>6.0869565217391312E-7</v>
       </c>
     </row>
     <row r="43" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D43">
         <v>4.3</v>
       </c>
-      <c r="E43" s="3">
-        <f t="shared" si="4"/>
-        <v>1.34375</v>
-      </c>
-      <c r="F43" s="3">
-        <f t="shared" si="5"/>
-        <v>2.5481481481481478</v>
+      <c r="E43">
+        <f t="shared" si="4"/>
+        <v>1.371014492753623</v>
+      </c>
+      <c r="F43">
+        <f t="shared" si="5"/>
+        <v>2.9975295381310416</v>
       </c>
       <c r="G43" s="1">
         <f t="shared" si="6"/>
-        <v>1.3437499999999998E-6</v>
+        <v>6.2318840579710141E-7</v>
       </c>
     </row>
     <row r="44" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D44">
         <v>4.4000000000000004</v>
       </c>
-      <c r="E44" s="3">
-        <f t="shared" si="4"/>
-        <v>1.375</v>
-      </c>
-      <c r="F44" s="3">
-        <f t="shared" si="5"/>
-        <v>2.6074074074074076</v>
+      <c r="E44">
+        <f t="shared" si="4"/>
+        <v>1.4028985507246376</v>
+      </c>
+      <c r="F44">
+        <f t="shared" si="5"/>
+        <v>3.0672395273899036</v>
       </c>
       <c r="G44" s="1">
         <f t="shared" si="6"/>
-        <v>1.3750000000000002E-6</v>
+        <v>6.3768115942028991E-7</v>
       </c>
     </row>
     <row r="45" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D45">
         <v>4.5</v>
       </c>
-      <c r="E45" s="3">
-        <f t="shared" si="4"/>
-        <v>1.40625</v>
-      </c>
-      <c r="F45" s="3">
-        <f t="shared" si="5"/>
-        <v>2.6666666666666665</v>
+      <c r="E45">
+        <f t="shared" si="4"/>
+        <v>1.4347826086956521</v>
+      </c>
+      <c r="F45">
+        <f t="shared" si="5"/>
+        <v>3.1369495166487646</v>
       </c>
       <c r="G45" s="1">
         <f t="shared" si="6"/>
-        <v>1.4062500000000001E-6</v>
+        <v>6.5217391304347831E-7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>